<commit_message>
Fazendo algumas mudanças necessárias.
</commit_message>
<xml_diff>
--- a/Faculdade/Disciplinas-Regulares/4-Ano/Gerenciamento_de_Configuracao_de_Software/Atividades/Atividades_Regulares/Planos_de_Mitigacao_Reducao_de_Probabilidade_e_Impacto_de_Riscos.xlsx
+++ b/Faculdade/Disciplinas-Regulares/4-Ano/Gerenciamento_de_Configuracao_de_Software/Atividades/Atividades_Regulares/Planos_de_Mitigacao_Reducao_de_Probabilidade_e_Impacto_de_Riscos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a473553081afb0a/Documentos/Pessoal/Estudos/Faculdade/Disciplinas Regulares/4º Ano/Gerenciamento de Configuração de Software/Atividades/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Estudos\Faculdade\Disciplinas-Regulares\4-Ano\Gerenciamento_de_Configuracao_de_Software\Atividades\Atividades_Regulares\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="8_{D2A53D12-8AFB-453F-8568-70D89122A3A9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{D064347D-0460-461B-A260-92D5192CD22E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE841A5-2EC4-46E6-B19F-2AFDC95C1092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F5277CAF-94F0-4ADE-8DE4-9D7834DE1D06}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
   <si>
     <t>Id</t>
   </si>
@@ -99,39 +99,18 @@
     <t>Plano de Redução de Impacto de Risco</t>
   </si>
   <si>
-    <t>Atraso no desenvolvimento da ideia do projeto.</t>
-  </si>
-  <si>
     <t>Estagnação no projeto, causando atrasos de entrega.</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>Atraso na realização de entrevista com possíveis usuários do aplicativo para levantamento de requisitos.</t>
-  </si>
-  <si>
     <t>Agendar entrevistas futuras com outros possíveis usuários afim de evitar a impossibilidade da realização da entrevista.</t>
   </si>
   <si>
-    <t>Falta de tempo hábil para prototipagem do projeto.</t>
-  </si>
-  <si>
     <t>Estagnação do projeto.</t>
   </si>
   <si>
-    <t>Atraso na realização do projeto.</t>
-  </si>
-  <si>
-    <t>Agenda desorganizada e rotina desregulada por parte do responsável pela prototipagem do modelo.</t>
-  </si>
-  <si>
-    <t>Alinhar a rtorina e agenda do responsável pela prototipagem do modelo de modo que haja tempo hábil para realização de tal tarefa, também garantindo que o mesmo não fique sobrecarregado com seus demais afazeres.</t>
-  </si>
-  <si>
-    <t>Fazer com que o tempo hábil para a realização da tarefa seja aproveitado da melhor forma, evitando pertubações e distrações.</t>
-  </si>
-  <si>
     <t>Pouca ou nenhuma referência na elaboração teórica do projeto.</t>
   </si>
   <si>
@@ -171,20 +150,56 @@
     <t>DEV3</t>
   </si>
   <si>
-    <t>PRO1</t>
-  </si>
-  <si>
     <t>ENG1</t>
   </si>
   <si>
     <t>ENG2</t>
+  </si>
+  <si>
+    <t>Requisitos do projeto não implementados de maneira correta.</t>
+  </si>
+  <si>
+    <t>Aplicativo final incondizente com o esperado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interesse do usuário e qualidade do produto baixos. </t>
+  </si>
+  <si>
+    <t>Pouca ou nenhuma implementação de atividades de verificação, afim de certificar que a documentação do projeto está englobando todos os requisitos.</t>
+  </si>
+  <si>
+    <t>Implementar atividades de verificação, afim de revisar a documentação, especificar o sistema e previnir falhas futuras.</t>
+  </si>
+  <si>
+    <t>Retrabalho na tarefa de levantamento de requisito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estagnação do projeto em sua fase de levantamento de requisitos, impossibilitando o início da fase de desenvolvimento. </t>
+  </si>
+  <si>
+    <t>Pouco ou nenhum backup dos arquivos de prototipagem do projeto.</t>
+  </si>
+  <si>
+    <t>Perda parcial ou total do progresso na etapa de prototipação.</t>
+  </si>
+  <si>
+    <t>Ausência de processos de backup dos arquivos de prototipagem.</t>
+  </si>
+  <si>
+    <t>Implementar processos e rotinas de backup, no qual haja redundância dos arquivos.</t>
+  </si>
+  <si>
+    <t>Os processos de backup devem ser feitos de maneira automática, com os arquivos copiados em um repositório, além de suas versões locais.</t>
+  </si>
+  <si>
+    <t>PROJ1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,11 +214,23 @@
       <family val="1"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -220,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -244,19 +271,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -264,17 +278,6 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -305,17 +308,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -343,45 +335,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="30">
     <dxf>
       <font>
         <b val="0"/>
@@ -395,27 +388,28 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -431,27 +425,30 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
         <right style="thin">
           <color auto="1"/>
         </right>
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -467,10 +464,11 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="13" formatCode="0%"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -482,7 +480,9 @@
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -504,8 +504,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -543,8 +543,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -564,44 +564,6 @@
         <top style="thin">
           <color auto="1"/>
         </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <bottom style="thin">
           <color auto="1"/>
         </bottom>
@@ -620,8 +582,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -630,6 +592,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color auto="1"/>
@@ -637,8 +600,12 @@
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -654,22 +621,23 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -677,7 +645,36 @@
           <color auto="1"/>
         </bottom>
         <vertical/>
-        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -693,33 +690,17 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -734,62 +715,25 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color auto="1"/>
         </left>
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -805,8 +749,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -815,15 +759,18 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color auto="1"/>
         </left>
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
         <bottom/>
+        <vertical/>
       </border>
     </dxf>
     <dxf>
@@ -839,8 +786,40 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom/>
+        <vertical/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -849,19 +828,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -876,8 +842,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -886,7 +852,6 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color auto="1"/>
@@ -894,12 +859,8 @@
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -915,11 +876,10 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="13" formatCode="0%"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -931,9 +891,7 @@
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
+        <right/>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -955,8 +913,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -994,8 +952,8 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -1019,6 +977,19 @@
           <color auto="1"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1033,17 +1004,16 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color auto="1"/>
@@ -1051,12 +1021,8 @@
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -1072,44 +1038,22 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color auto="1"/>
         </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
+        <right/>
         <top style="thin">
           <color auto="1"/>
         </top>
@@ -1131,20 +1075,27 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
         <bottom style="thin">
           <color auto="1"/>
         </bottom>
@@ -1163,16 +1114,17 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color auto="1"/>
@@ -1180,8 +1132,72 @@
         <right style="thin">
           <color auto="1"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
       </border>
     </dxf>
   </dxfs>
@@ -1198,39 +1214,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC38A7DD-DBEA-4DC8-A9A0-43687E2E62F6}" name="Mitigação" displayName="Mitigação" ref="A3:G8" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25" totalsRowBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC38A7DD-DBEA-4DC8-A9A0-43687E2E62F6}" name="Mitigação" displayName="Mitigação" ref="B4:H9" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C27E8E9C-675C-48D0-B052-1C0DEF01345F}" name="Id" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{C1B38B78-E9CE-40ED-A9F2-8BAA2B0BC129}" name="Causa" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{E2961184-1CA4-41F6-A37A-BCADE58C500C}" name="Risco" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{77A98E45-A829-43BD-B115-38CF2E3CFF34}" name="Efeito" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{6274A4CE-EA3C-4CEE-B720-C607D47F5712}" name="Prob." dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{CEFE2CB2-E460-4BCD-9702-F35E56359D11}" name="Imp." dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{40F5FDF0-5956-4862-9115-10EB4A94BD62}" name="Exp." dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{C27E8E9C-675C-48D0-B052-1C0DEF01345F}" name="Id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{C1B38B78-E9CE-40ED-A9F2-8BAA2B0BC129}" name="Causa" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{E2961184-1CA4-41F6-A37A-BCADE58C500C}" name="Risco" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{77A98E45-A829-43BD-B115-38CF2E3CFF34}" name="Efeito" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{6274A4CE-EA3C-4CEE-B720-C607D47F5712}" name="Prob." dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{CEFE2CB2-E460-4BCD-9702-F35E56359D11}" name="Imp." dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{40F5FDF0-5956-4862-9115-10EB4A94BD62}" name="Exp." dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F896D628-C6ED-4CCE-BF13-427E739F89D2}" name="Probabilidade" displayName="Probabilidade" ref="A12:D17" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F896D628-C6ED-4CCE-BF13-427E739F89D2}" name="Probabilidade" displayName="Probabilidade" ref="B13:E18" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" headerRowBorderDxfId="29" tableBorderDxfId="28" totalsRowBorderDxfId="27">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{97CF8E47-2442-407D-A592-6337CC52E7CB}" name="Id" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{26D772EE-73C9-4F3C-89FE-1D8C8FEE4512}" name="Causa do Risco" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{86BCF522-17DE-407A-A597-36C90FB600F3}" name="Risco" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{C695896E-D2DA-4DA1-AF69-890CA41FC964}" name="Plano de redução de probabilidade" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{97CF8E47-2442-407D-A592-6337CC52E7CB}" name="Id" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{26D772EE-73C9-4F3C-89FE-1D8C8FEE4512}" name="Causa do Risco" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{86BCF522-17DE-407A-A597-36C90FB600F3}" name="Risco" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{C695896E-D2DA-4DA1-AF69-890CA41FC964}" name="Plano de redução de probabilidade" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B71494D1-6001-4AE8-A663-71239ACE4032}" name="Impacto" displayName="Impacto" ref="A21:D26" totalsRowShown="0" headerRowDxfId="9" dataDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B71494D1-6001-4AE8-A663-71239ACE4032}" name="Impacto" displayName="Impacto" ref="B22:E27" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" headerRowBorderDxfId="26" tableBorderDxfId="25" totalsRowBorderDxfId="24">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{28C0BE72-78D4-48E1-8721-683CBFD7C963}" name="Id" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{85B230AD-ABAD-437F-B9AC-676682155473}" name="Risco" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{32B394CD-38A9-408E-B33C-5C3B80FCA185}" name="Efeito" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{0EB5FDB1-80CA-48F8-81E4-8264D7959D8A}" name="Plano de redução de impacto" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{28C0BE72-78D4-48E1-8721-683CBFD7C963}" name="Id" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{85B230AD-ABAD-437F-B9AC-676682155473}" name="Risco" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{32B394CD-38A9-408E-B33C-5C3B80FCA185}" name="Efeito" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{0EB5FDB1-80CA-48F8-81E4-8264D7959D8A}" name="Plano de redução de impacto" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1533,501 +1549,528 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D5B45C8-4507-4342-BD8E-4B38EAB88ABB}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="B2:I34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" style="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="57.6640625" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.88671875" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="58.44140625" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.21875" style="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.44140625" style="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="18"/>
+    <col min="1" max="1" width="8.88671875" style="2"/>
+    <col min="2" max="2" width="8.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="43.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="58.44140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.21875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="7.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="7.44140625" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1"/>
-      <c r="B1" s="6" t="s">
+    <row r="2" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B2" s="3"/>
+      <c r="C2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="5"/>
+    </row>
+    <row r="4" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H4" s="7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B5" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B9" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B11" s="14"/>
+      <c r="C11" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="14"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B13" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="5"/>
+    </row>
+    <row r="14" spans="2:9" ht="60.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="5"/>
+    </row>
+    <row r="15" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="D15" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="5"/>
+    </row>
+    <row r="16" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B17" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="5"/>
+    </row>
+    <row r="18" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="5"/>
+    </row>
+    <row r="20" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="14"/>
+      <c r="C20" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="14"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="5"/>
+    </row>
+    <row r="21" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="5"/>
+    </row>
+    <row r="22" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B22" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="5"/>
+    </row>
+    <row r="23" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="12" t="s">
+      <c r="D23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="5"/>
+    </row>
+    <row r="24" spans="2:9" ht="60.6" x14ac:dyDescent="0.3">
+      <c r="B24" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="15" t="s">
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="5"/>
+    </row>
+    <row r="25" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B25" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="E25" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="5"/>
+    </row>
+    <row r="26" spans="2:9" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="15" t="s">
+      <c r="E26" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="5"/>
+    </row>
+    <row r="27" spans="2:9" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="B27" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="D27" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-    </row>
-    <row r="23" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-    </row>
-    <row r="24" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-    </row>
-    <row r="25" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-    </row>
-    <row r="26" spans="1:7" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-    </row>
-    <row r="27" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-    </row>
-    <row r="28" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="5"/>
+    </row>
+    <row r="28" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
-    </row>
-    <row r="29" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-    </row>
-    <row r="30" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
-    </row>
-    <row r="31" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
-    </row>
-    <row r="32" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
+      <c r="H31" s="1"/>
+    </row>
+    <row r="32" spans="2:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
-    </row>
-    <row r="33" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+    </row>
+    <row r="34" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>